<commit_message>
Sync local work: dashboard, boletín, docs, SRI (renta/DINA, movilidad), actas y datos
- Automatización: scripts Stata/R y datasets dashboard (significancia, NBI test)
- Boletín 2: análisis mortalidad, reorganización materno-infantil, nuevas carpetas
- Dashboards: Excel actualizados, NBI, PDF mercado laboral
- docs: actualización frontend dashboard
- SRI: actas, scripts renta/DINA y movilidad, resultados (gráficos, matriz transición)
- Elimina gráficos boletín y archivo 05_mort_materna_infantil sin extensión

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Dashboards/Data final/empleo_demografico.xlsx
+++ b/Dashboards/Data final/empleo_demografico.xlsx
@@ -391,7 +391,7 @@
         </is>
       </c>
       <c r="D2">
-        <v>23.57499178228778</v>
+        <v>23.7496389187056</v>
       </c>
     </row>
     <row r="3">
@@ -409,7 +409,7 @@
         </is>
       </c>
       <c r="D3">
-        <v>52.41503830112557</v>
+        <v>52.89895901930952</v>
       </c>
     </row>
     <row r="4">
@@ -427,7 +427,7 @@
         </is>
       </c>
       <c r="D4">
-        <v>25.13627900914169</v>
+        <v>25.25918302630837</v>
       </c>
     </row>
     <row r="5">
@@ -445,7 +445,7 @@
         </is>
       </c>
       <c r="D5">
-        <v>53.56239148275469</v>
+        <v>54.03326711139537</v>
       </c>
     </row>
     <row r="6">
@@ -463,7 +463,7 @@
         </is>
       </c>
       <c r="D6">
-        <v>21.48530290037948</v>
+        <v>21.61864459952175</v>
       </c>
     </row>
     <row r="7">
@@ -481,7 +481,7 @@
         </is>
       </c>
       <c r="D7">
-        <v>47.302137700349</v>
+        <v>47.76798231859861</v>
       </c>
     </row>
     <row r="8">
@@ -499,7 +499,7 @@
         </is>
       </c>
       <c r="D8">
-        <v>25.79222516434923</v>
+        <v>25.91918901838237</v>
       </c>
     </row>
     <row r="9">
@@ -517,7 +517,7 @@
         </is>
       </c>
       <c r="D9">
-        <v>53.57862968581839</v>
+        <v>53.87024008654304</v>
       </c>
     </row>
     <row r="10">
@@ -535,7 +535,7 @@
         </is>
       </c>
       <c r="D10">
-        <v>24.81384429596542</v>
+        <v>25.00076933478186</v>
       </c>
     </row>
     <row r="11">
@@ -553,7 +553,7 @@
         </is>
       </c>
       <c r="D11">
-        <v>55.18426241391155</v>
+        <v>55.45178010041661</v>
       </c>
     </row>
     <row r="12">
@@ -571,7 +571,7 @@
         </is>
       </c>
       <c r="D12">
-        <v>25.83932927398251</v>
+        <v>26.00356046671155</v>
       </c>
     </row>
     <row r="13">
@@ -589,7 +589,7 @@
         </is>
       </c>
       <c r="D13">
-        <v>56.27751316202809</v>
+        <v>56.54393947298607</v>
       </c>
     </row>
     <row r="14">
@@ -607,7 +607,7 @@
         </is>
       </c>
       <c r="D14">
-        <v>28.70662432439542</v>
+        <v>28.85027180224976</v>
       </c>
     </row>
     <row r="15">
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="D15">
-        <v>56.55667583581317</v>
+        <v>56.91946403489867</v>
       </c>
     </row>
     <row r="16">
@@ -643,7 +643,7 @@
         </is>
       </c>
       <c r="D16">
-        <v>34.12542832166704</v>
+        <v>34.40569441536054</v>
       </c>
     </row>
     <row r="17">
@@ -661,7 +661,7 @@
         </is>
       </c>
       <c r="D17">
-        <v>55.97682087920123</v>
+        <v>56.39132645893395</v>
       </c>
     </row>
     <row r="18">
@@ -679,7 +679,7 @@
         </is>
       </c>
       <c r="D18">
-        <v>30.00103422438448</v>
+        <v>30.17913188471564</v>
       </c>
     </row>
     <row r="19">
@@ -697,7 +697,7 @@
         </is>
       </c>
       <c r="D19">
-        <v>53.63942587910556</v>
+        <v>54.04085435863647</v>
       </c>
     </row>
     <row r="20">
@@ -715,7 +715,7 @@
         </is>
       </c>
       <c r="D20">
-        <v>27.4870432164044</v>
+        <v>27.7611436946131</v>
       </c>
     </row>
     <row r="21">
@@ -733,7 +733,7 @@
         </is>
       </c>
       <c r="D21">
-        <v>47.11114922032497</v>
+        <v>47.64220863703964</v>
       </c>
     </row>
     <row r="22">
@@ -751,7 +751,7 @@
         </is>
       </c>
       <c r="D22">
-        <v>24.97442931940399</v>
+        <v>25.1383666496709</v>
       </c>
     </row>
     <row r="23">
@@ -769,7 +769,7 @@
         </is>
       </c>
       <c r="D23">
-        <v>49.88302509509278</v>
+        <v>50.36524259609785</v>
       </c>
     </row>
     <row r="24">
@@ -787,7 +787,7 @@
         </is>
       </c>
       <c r="D24">
-        <v>22.83362139681021</v>
+        <v>23.03638831965663</v>
       </c>
     </row>
     <row r="25">
@@ -805,7 +805,7 @@
         </is>
       </c>
       <c r="D25">
-        <v>48.88109271126522</v>
+        <v>49.27718104414508</v>
       </c>
     </row>
     <row r="26">
@@ -823,7 +823,7 @@
         </is>
       </c>
       <c r="D26">
-        <v>20.50216064277741</v>
+        <v>20.64981377580154</v>
       </c>
     </row>
     <row r="27">
@@ -841,7 +841,7 @@
         </is>
       </c>
       <c r="D27">
-        <v>47.65979747692055</v>
+        <v>48.02205999923117</v>
       </c>
     </row>
     <row r="28">
@@ -859,7 +859,7 @@
         </is>
       </c>
       <c r="D28">
-        <v>17.5592971008419</v>
+        <v>17.74055679107208</v>
       </c>
     </row>
     <row r="29">
@@ -877,7 +877,7 @@
         </is>
       </c>
       <c r="D29">
-        <v>37.12278558111413</v>
+        <v>37.44425281397636</v>
       </c>
     </row>
     <row r="30">
@@ -895,7 +895,7 @@
         </is>
       </c>
       <c r="D30">
-        <v>19.69293670760913</v>
+        <v>20.02176022746248</v>
       </c>
     </row>
     <row r="31">
@@ -913,7 +913,7 @@
         </is>
       </c>
       <c r="D31">
-        <v>40.65504921879145</v>
+        <v>40.99182550046679</v>
       </c>
     </row>
     <row r="32">
@@ -931,7 +931,7 @@
         </is>
       </c>
       <c r="D32">
-        <v>19.96843053420861</v>
+        <v>19.98893512699535</v>
       </c>
     </row>
     <row r="33">
@@ -949,7 +949,7 @@
         </is>
       </c>
       <c r="D33">
-        <v>44.25807853934212</v>
+        <v>44.5266313328913</v>
       </c>
     </row>
     <row r="34">
@@ -967,7 +967,7 @@
         </is>
       </c>
       <c r="D34">
-        <v>18.15694471985556</v>
+        <v>18.13795678359173</v>
       </c>
     </row>
     <row r="35">
@@ -985,7 +985,7 @@
         </is>
       </c>
       <c r="D35">
-        <v>45.00572006146763</v>
+        <v>45.27396755371329</v>
       </c>
     </row>
     <row r="36">
@@ -1003,7 +1003,7 @@
         </is>
       </c>
       <c r="D36">
-        <v>17.69531538467068</v>
+        <v>17.72116203398426</v>
       </c>
     </row>
     <row r="37">
@@ -1021,7 +1021,7 @@
         </is>
       </c>
       <c r="D37">
-        <v>41.30250417913693</v>
+        <v>41.53197332393969</v>
       </c>
     </row>
     <row r="38">
@@ -1039,7 +1039,7 @@
         </is>
       </c>
       <c r="D38">
-        <v>50.05288408206339</v>
+        <v>50.49779872490456</v>
       </c>
     </row>
     <row r="39">
@@ -1057,7 +1057,7 @@
         </is>
       </c>
       <c r="D39">
-        <v>32.1389516601177</v>
+        <v>32.42562358471615</v>
       </c>
     </row>
     <row r="40">
@@ -1075,7 +1075,7 @@
         </is>
       </c>
       <c r="D40">
-        <v>51.9540819038307</v>
+        <v>52.39139209357911</v>
       </c>
     </row>
     <row r="41">
@@ -1093,7 +1093,7 @@
         </is>
       </c>
       <c r="D41">
-        <v>33.3168017498204</v>
+        <v>33.56024930453227</v>
       </c>
     </row>
     <row r="42">
@@ -1111,7 +1111,7 @@
         </is>
       </c>
       <c r="D42">
-        <v>44.88859293798257</v>
+        <v>45.24929592049104</v>
       </c>
     </row>
     <row r="43">
@@ -1129,7 +1129,7 @@
         </is>
       </c>
       <c r="D43">
-        <v>29.87736151233486</v>
+        <v>30.22792446786651</v>
       </c>
     </row>
     <row r="44">
@@ -1147,7 +1147,7 @@
         </is>
       </c>
       <c r="D44">
-        <v>49.79469853803195</v>
+        <v>50.03134804279957</v>
       </c>
     </row>
     <row r="45">
@@ -1165,7 +1165,7 @@
         </is>
       </c>
       <c r="D45">
-        <v>36.20995655984213</v>
+        <v>36.44863311665794</v>
       </c>
     </row>
     <row r="46">
@@ -1183,7 +1183,7 @@
         </is>
       </c>
       <c r="D46">
-        <v>51.53749248324433</v>
+        <v>51.83984777107917</v>
       </c>
     </row>
     <row r="47">
@@ -1201,7 +1201,7 @@
         </is>
       </c>
       <c r="D47">
-        <v>35.74865783674797</v>
+        <v>35.89666331325766</v>
       </c>
     </row>
     <row r="48">
@@ -1219,7 +1219,7 @@
         </is>
       </c>
       <c r="D48">
-        <v>51.33340497784054</v>
+        <v>51.57186232963176</v>
       </c>
     </row>
     <row r="49">
@@ -1237,7 +1237,7 @@
         </is>
       </c>
       <c r="D49">
-        <v>38.6638151174668</v>
+        <v>38.88834645196179</v>
       </c>
     </row>
     <row r="50">
@@ -1255,7 +1255,7 @@
         </is>
       </c>
       <c r="D50">
-        <v>53.26602873377728</v>
+        <v>53.52029441888956</v>
       </c>
     </row>
     <row r="51">
@@ -1273,7 +1273,7 @@
         </is>
       </c>
       <c r="D51">
-        <v>38.79526730431611</v>
+        <v>39.1456613605568</v>
       </c>
     </row>
     <row r="52">
@@ -1291,7 +1291,7 @@
         </is>
       </c>
       <c r="D52">
-        <v>55.78358976911129</v>
+        <v>56.19184207019614</v>
       </c>
     </row>
     <row r="53">
@@ -1309,7 +1309,7 @@
         </is>
       </c>
       <c r="D53">
-        <v>38.70573976039819</v>
+        <v>39.02167085535649</v>
       </c>
     </row>
     <row r="54">
@@ -1327,7 +1327,7 @@
         </is>
       </c>
       <c r="D54">
-        <v>52.77204247784745</v>
+        <v>53.09746671889525</v>
       </c>
     </row>
     <row r="55">
@@ -1345,7 +1345,7 @@
         </is>
       </c>
       <c r="D55">
-        <v>36.5540018684441</v>
+        <v>36.89282529916569</v>
       </c>
     </row>
     <row r="56">
@@ -1363,7 +1363,7 @@
         </is>
       </c>
       <c r="D56">
-        <v>47.43944712210115</v>
+        <v>47.8971736169321</v>
       </c>
     </row>
     <row r="57">
@@ -1381,7 +1381,7 @@
         </is>
       </c>
       <c r="D57">
-        <v>31.42202406006087</v>
+        <v>31.85565056730701</v>
       </c>
     </row>
     <row r="58">
@@ -1399,7 +1399,7 @@
         </is>
       </c>
       <c r="D58">
-        <v>49.09185937074098</v>
+        <v>49.50938248408681</v>
       </c>
     </row>
     <row r="59">
@@ -1417,7 +1417,7 @@
         </is>
       </c>
       <c r="D59">
-        <v>32.0489970890068</v>
+        <v>32.37781796862092</v>
       </c>
     </row>
     <row r="60">
@@ -1435,7 +1435,7 @@
         </is>
       </c>
       <c r="D60">
-        <v>46.09862961225916</v>
+        <v>46.45721721263138</v>
       </c>
     </row>
     <row r="61">
@@ -1453,7 +1453,7 @@
         </is>
       </c>
       <c r="D61">
-        <v>32.16911654587997</v>
+        <v>32.46483328081738</v>
       </c>
     </row>
     <row r="62">
@@ -1471,7 +1471,7 @@
         </is>
       </c>
       <c r="D62">
-        <v>44.51824591509285</v>
+        <v>44.80888430300161</v>
       </c>
     </row>
     <row r="63">
@@ -1489,7 +1489,7 @@
         </is>
       </c>
       <c r="D63">
-        <v>30.26622594840928</v>
+        <v>30.55614109361189</v>
       </c>
     </row>
     <row r="64">
@@ -1507,7 +1507,7 @@
         </is>
       </c>
       <c r="D64">
-        <v>35.52848134407698</v>
+        <v>35.81376553337925</v>
       </c>
     </row>
     <row r="65">
@@ -1525,7 +1525,7 @@
         </is>
       </c>
       <c r="D65">
-        <v>23.6113258255937</v>
+        <v>23.87074716675982</v>
       </c>
     </row>
     <row r="66">
@@ -1543,7 +1543,7 @@
         </is>
       </c>
       <c r="D66">
-        <v>38.62820148414789</v>
+        <v>38.94734453653147</v>
       </c>
     </row>
     <row r="67">
@@ -1561,7 +1561,7 @@
         </is>
       </c>
       <c r="D67">
-        <v>26.8479112536787</v>
+        <v>27.20215145902838</v>
       </c>
     </row>
     <row r="68">
@@ -1579,7 +1579,7 @@
         </is>
       </c>
       <c r="D68">
-        <v>40.86378974611053</v>
+        <v>41.123593764622</v>
       </c>
     </row>
     <row r="69">
@@ -1597,7 +1597,7 @@
         </is>
       </c>
       <c r="D69">
-        <v>28.73490779593</v>
+        <v>28.80812424553461</v>
       </c>
     </row>
     <row r="70">
@@ -1615,7 +1615,7 @@
         </is>
       </c>
       <c r="D70">
-        <v>40.91981770137157</v>
+        <v>41.11873338444835</v>
       </c>
     </row>
     <row r="71">
@@ -1633,7 +1633,7 @@
         </is>
       </c>
       <c r="D71">
-        <v>28.62392643234575</v>
+        <v>28.75219846619985</v>
       </c>
     </row>
     <row r="72">
@@ -1651,7 +1651,7 @@
         </is>
       </c>
       <c r="D72">
-        <v>37.31546155824018</v>
+        <v>37.4053362534242</v>
       </c>
     </row>
     <row r="73">
@@ -1669,7 +1669,7 @@
         </is>
       </c>
       <c r="D73">
-        <v>26.40920401251958</v>
+        <v>26.66327334680922</v>
       </c>
     </row>
     <row r="74">
@@ -1687,7 +1687,7 @@
         </is>
       </c>
       <c r="D74">
-        <v>22.72819728918448</v>
+        <v>23.01604423104186</v>
       </c>
     </row>
     <row r="75">
@@ -1705,7 +1705,7 @@
         </is>
       </c>
       <c r="D75">
-        <v>44.41906740175238</v>
+        <v>44.80399463046446</v>
       </c>
     </row>
     <row r="76">
@@ -1723,7 +1723,7 @@
         </is>
       </c>
       <c r="D76">
-        <v>20.10206701099736</v>
+        <v>20.14971197387742</v>
       </c>
     </row>
     <row r="77">
@@ -1741,7 +1741,7 @@
         </is>
       </c>
       <c r="D77">
-        <v>46.08344381310519</v>
+        <v>46.45993018671496</v>
       </c>
     </row>
     <row r="78">
@@ -1759,7 +1759,7 @@
         </is>
       </c>
       <c r="D78">
-        <v>17.88961220877267</v>
+        <v>18.12161873317797</v>
       </c>
     </row>
     <row r="79">
@@ -1777,7 +1777,7 @@
         </is>
       </c>
       <c r="D79">
-        <v>40.41516992471526</v>
+        <v>40.7812702501477</v>
       </c>
     </row>
     <row r="80">
@@ -1795,7 +1795,7 @@
         </is>
       </c>
       <c r="D80">
-        <v>19.92540689655172</v>
+        <v>19.98918620689655</v>
       </c>
     </row>
     <row r="81">
@@ -1813,7 +1813,7 @@
         </is>
       </c>
       <c r="D81">
-        <v>46.13181403544605</v>
+        <v>46.38255703858077</v>
       </c>
     </row>
     <row r="82">
@@ -1831,7 +1831,7 @@
         </is>
       </c>
       <c r="D82">
-        <v>19.62551640140231</v>
+        <v>19.71830406372928</v>
       </c>
     </row>
     <row r="83">
@@ -1849,7 +1849,7 @@
         </is>
       </c>
       <c r="D83">
-        <v>47.1971062941914</v>
+        <v>47.45736234282067</v>
       </c>
     </row>
     <row r="84">
@@ -1867,7 +1867,7 @@
         </is>
       </c>
       <c r="D84">
-        <v>20.73497425700707</v>
+        <v>21.03255380836597</v>
       </c>
     </row>
     <row r="85">
@@ -1885,7 +1885,7 @@
         </is>
       </c>
       <c r="D85">
-        <v>48.02633385596539</v>
+        <v>48.25408091076591</v>
       </c>
     </row>
     <row r="86">
@@ -1903,7 +1903,7 @@
         </is>
       </c>
       <c r="D86">
-        <v>25.23012157285145</v>
+        <v>25.42687819970905</v>
       </c>
     </row>
     <row r="87">
@@ -1921,7 +1921,7 @@
         </is>
       </c>
       <c r="D87">
-        <v>49.07334574307342</v>
+        <v>49.36859286749687</v>
       </c>
     </row>
     <row r="88">
@@ -1939,7 +1939,7 @@
         </is>
       </c>
       <c r="D88">
-        <v>27.11333640345291</v>
+        <v>27.45451160603181</v>
       </c>
     </row>
     <row r="89">
@@ -1957,7 +1957,7 @@
         </is>
       </c>
       <c r="D89">
-        <v>50.56068712750814</v>
+        <v>50.93920145951759</v>
       </c>
     </row>
     <row r="90">
@@ -1975,7 +1975,7 @@
         </is>
       </c>
       <c r="D90">
-        <v>22.31403522354008</v>
+        <v>22.58641964580545</v>
       </c>
     </row>
     <row r="91">
@@ -1993,7 +1993,7 @@
         </is>
       </c>
       <c r="D91">
-        <v>48.46683746509354</v>
+        <v>48.79563311308021</v>
       </c>
     </row>
     <row r="92">
@@ -2011,7 +2011,7 @@
         </is>
       </c>
       <c r="D92">
-        <v>20.10207482285347</v>
+        <v>20.28151345498681</v>
       </c>
     </row>
     <row r="93">
@@ -2029,7 +2029,7 @@
         </is>
       </c>
       <c r="D93">
-        <v>42.66791285107813</v>
+        <v>43.13128802465584</v>
       </c>
     </row>
     <row r="94">
@@ -2047,7 +2047,7 @@
         </is>
       </c>
       <c r="D94">
-        <v>18.87845344492202</v>
+        <v>19.0062634945888</v>
       </c>
     </row>
     <row r="95">
@@ -2065,7 +2065,7 @@
         </is>
       </c>
       <c r="D95">
-        <v>44.28361924180514</v>
+        <v>44.69361752995017</v>
       </c>
     </row>
     <row r="96">
@@ -2083,7 +2083,7 @@
         </is>
       </c>
       <c r="D96">
-        <v>16.28910523162171</v>
+        <v>16.43711554424368</v>
       </c>
     </row>
     <row r="97">
@@ -2101,7 +2101,7 @@
         </is>
       </c>
       <c r="D97">
-        <v>42.65256469039382</v>
+        <v>42.99474458873377</v>
       </c>
     </row>
     <row r="98">
@@ -2119,7 +2119,7 @@
         </is>
       </c>
       <c r="D98">
-        <v>14.96355451337809</v>
+        <v>15.06664159541639</v>
       </c>
     </row>
     <row r="99">
@@ -2137,7 +2137,7 @@
         </is>
       </c>
       <c r="D99">
-        <v>41.39842399333217</v>
+        <v>41.71382599486799</v>
       </c>
     </row>
     <row r="100">
@@ -2155,7 +2155,7 @@
         </is>
       </c>
       <c r="D100">
-        <v>10.48517454046929</v>
+        <v>10.49083959951809</v>
       </c>
     </row>
     <row r="101">
@@ -2173,7 +2173,7 @@
         </is>
       </c>
       <c r="D101">
-        <v>33.54543189527953</v>
+        <v>33.84447184619271</v>
       </c>
     </row>
     <row r="102">
@@ -2191,7 +2191,7 @@
         </is>
       </c>
       <c r="D102">
-        <v>13.88016170624866</v>
+        <v>14.16628191990511</v>
       </c>
     </row>
     <row r="103">
@@ -2209,7 +2209,7 @@
         </is>
       </c>
       <c r="D103">
-        <v>36.21767061121633</v>
+        <v>36.55252564496895</v>
       </c>
     </row>
     <row r="104">
@@ -2227,7 +2227,7 @@
         </is>
       </c>
       <c r="D104">
-        <v>13.47519544646681</v>
+        <v>13.506743518908</v>
       </c>
     </row>
     <row r="105">
@@ -2245,7 +2245,7 @@
         </is>
       </c>
       <c r="D105">
-        <v>39.06239833116324</v>
+        <v>39.26876491574654</v>
       </c>
     </row>
     <row r="106">
@@ -2263,7 +2263,7 @@
         </is>
       </c>
       <c r="D106">
-        <v>13.45660981625206</v>
+        <v>13.55099840271659</v>
       </c>
     </row>
     <row r="107">
@@ -2281,7 +2281,7 @@
         </is>
       </c>
       <c r="D107">
-        <v>39.38070793274426</v>
+        <v>39.56360250329763</v>
       </c>
     </row>
     <row r="108">
@@ -2299,7 +2299,7 @@
         </is>
       </c>
       <c r="D108">
-        <v>11.73874872791895</v>
+        <v>11.79160654343302</v>
       </c>
     </row>
     <row r="109">
@@ -2317,7 +2317,7 @@
         </is>
       </c>
       <c r="D109">
-        <v>37.79622261016659</v>
+        <v>37.96865689116763</v>
       </c>
     </row>
     <row r="110">
@@ -2335,7 +2335,7 @@
         </is>
       </c>
       <c r="D110">
-        <v>36.77703505650526</v>
+        <v>37.14147024195633</v>
       </c>
     </row>
     <row r="111">
@@ -2353,7 +2353,7 @@
         </is>
       </c>
       <c r="D111">
-        <v>67.36220702087181</v>
+        <v>67.81055008521794</v>
       </c>
     </row>
     <row r="112">
@@ -2371,7 +2371,7 @@
         </is>
       </c>
       <c r="D112">
-        <v>37.7064213721472</v>
+        <v>37.9862673365387</v>
       </c>
     </row>
     <row r="113">
@@ -2389,7 +2389,7 @@
         </is>
       </c>
       <c r="D113">
-        <v>71.29110952260264</v>
+        <v>71.96670514135329</v>
       </c>
     </row>
     <row r="114">
@@ -2407,7 +2407,7 @@
         </is>
       </c>
       <c r="D114">
-        <v>33.04329741598641</v>
+        <v>33.35989998858951</v>
       </c>
     </row>
     <row r="115">
@@ -2425,7 +2425,7 @@
         </is>
       </c>
       <c r="D115">
-        <v>60.84563740634158</v>
+        <v>61.35475118974482</v>
       </c>
     </row>
     <row r="116">
@@ -2443,7 +2443,7 @@
         </is>
       </c>
       <c r="D116">
-        <v>37.52113757118768</v>
+        <v>37.77341637237123</v>
       </c>
     </row>
     <row r="117">
@@ -2461,7 +2461,7 @@
         </is>
       </c>
       <c r="D117">
-        <v>69.16182050017271</v>
+        <v>69.34626149824372</v>
       </c>
     </row>
     <row r="118">
@@ -2479,7 +2479,7 @@
         </is>
       </c>
       <c r="D118">
-        <v>38.15199555174733</v>
+        <v>38.35430177279947</v>
       </c>
     </row>
     <row r="119">
@@ -2497,7 +2497,7 @@
         </is>
       </c>
       <c r="D119">
-        <v>71.01839882814113</v>
+        <v>71.40010679984687</v>
       </c>
     </row>
     <row r="120">
@@ -2515,7 +2515,7 @@
         </is>
       </c>
       <c r="D120">
-        <v>39.34715035910109</v>
+        <v>39.55560274924705</v>
       </c>
     </row>
     <row r="121">
@@ -2533,7 +2533,7 @@
         </is>
       </c>
       <c r="D121">
-        <v>69.96105768535715</v>
+        <v>70.27727506311862</v>
       </c>
     </row>
     <row r="122">
@@ -2551,7 +2551,7 @@
         </is>
       </c>
       <c r="D122">
-        <v>39.75673417538135</v>
+        <v>39.92317281067302</v>
       </c>
     </row>
     <row r="123">
@@ -2569,7 +2569,7 @@
         </is>
       </c>
       <c r="D123">
-        <v>75.3356953856167</v>
+        <v>76.07416957667056</v>
       </c>
     </row>
     <row r="124">
@@ -2587,7 +2587,7 @@
         </is>
       </c>
       <c r="D124">
-        <v>42.2116183643809</v>
+        <v>42.5477818997775</v>
       </c>
     </row>
     <row r="125">
@@ -2605,7 +2605,7 @@
         </is>
       </c>
       <c r="D125">
-        <v>75.20218418450611</v>
+        <v>75.71039027244143</v>
       </c>
     </row>
     <row r="126">
@@ -2623,7 +2623,7 @@
         </is>
       </c>
       <c r="D126">
-        <v>39.18337196262701</v>
+        <v>39.45921032730662</v>
       </c>
     </row>
     <row r="127">
@@ -2641,7 +2641,7 @@
         </is>
       </c>
       <c r="D127">
-        <v>71.38062363032151</v>
+        <v>71.91003297365609</v>
       </c>
     </row>
     <row r="128">
@@ -2659,7 +2659,7 @@
         </is>
       </c>
       <c r="D128">
-        <v>33.76206804660586</v>
+        <v>34.11462998815269</v>
       </c>
     </row>
     <row r="129">
@@ -2677,7 +2677,7 @@
         </is>
       </c>
       <c r="D129">
-        <v>67.17196036444862</v>
+        <v>67.97972502197854</v>
       </c>
     </row>
     <row r="130">
@@ -2695,7 +2695,7 @@
         </is>
       </c>
       <c r="D130">
-        <v>34.82222985310447</v>
+        <v>35.10642035677862</v>
       </c>
     </row>
     <row r="131">
@@ -2713,7 +2713,7 @@
         </is>
       </c>
       <c r="D131">
-        <v>68.76236211487257</v>
+        <v>69.50706066945607</v>
       </c>
     </row>
     <row r="132">
@@ -2731,7 +2731,7 @@
         </is>
       </c>
       <c r="D132">
-        <v>33.0321683065395</v>
+        <v>33.29721216384701</v>
       </c>
     </row>
     <row r="133">
@@ -2749,7 +2749,7 @@
         </is>
       </c>
       <c r="D133">
-        <v>68.22462975320094</v>
+        <v>68.81578289061648</v>
       </c>
     </row>
     <row r="134">
@@ -2767,7 +2767,7 @@
         </is>
       </c>
       <c r="D134">
-        <v>31.59781046175004</v>
+        <v>31.82251623125869</v>
       </c>
     </row>
     <row r="135">
@@ -2785,7 +2785,7 @@
         </is>
       </c>
       <c r="D135">
-        <v>65.210907401809</v>
+        <v>65.75256862741591</v>
       </c>
     </row>
     <row r="136">
@@ -2803,7 +2803,7 @@
         </is>
       </c>
       <c r="D136">
-        <v>23.98729695134267</v>
+        <v>24.13597831999812</v>
       </c>
     </row>
     <row r="137">
@@ -2821,7 +2821,7 @@
         </is>
       </c>
       <c r="D137">
-        <v>56.59608816529554</v>
+        <v>57.36784354619486</v>
       </c>
     </row>
     <row r="138">
@@ -2839,7 +2839,7 @@
         </is>
       </c>
       <c r="D138">
-        <v>26.30795203311723</v>
+        <v>26.54416291721701</v>
       </c>
     </row>
     <row r="139">
@@ -2857,7 +2857,7 @@
         </is>
       </c>
       <c r="D139">
-        <v>60.20563282351596</v>
+        <v>60.89645589464205</v>
       </c>
     </row>
     <row r="140">
@@ -2875,7 +2875,7 @@
         </is>
       </c>
       <c r="D140">
-        <v>27.99812582138163</v>
+        <v>28.14574405272079</v>
       </c>
     </row>
     <row r="141">
@@ -2893,7 +2893,7 @@
         </is>
       </c>
       <c r="D141">
-        <v>64.57594141140392</v>
+        <v>64.8870150304889</v>
       </c>
     </row>
     <row r="142">
@@ -2911,7 +2911,7 @@
         </is>
       </c>
       <c r="D142">
-        <v>27.81330644431958</v>
+        <v>27.92208107319987</v>
       </c>
     </row>
     <row r="143">
@@ -2929,7 +2929,7 @@
         </is>
       </c>
       <c r="D143">
-        <v>65.50115148921527</v>
+        <v>65.89694833298773</v>
       </c>
     </row>
     <row r="144">
@@ -2947,7 +2947,7 @@
         </is>
       </c>
       <c r="D144">
-        <v>25.86010656668527</v>
+        <v>25.90620360281551</v>
       </c>
     </row>
     <row r="145">
@@ -2965,7 +2965,7 @@
         </is>
       </c>
       <c r="D145">
-        <v>63.06183626490416</v>
+        <v>63.69498623708121</v>
       </c>
     </row>
     <row r="146">
@@ -2983,7 +2983,7 @@
         </is>
       </c>
       <c r="D146">
-        <v>48.5237001385736</v>
+        <v>48.95856768829409</v>
       </c>
     </row>
     <row r="147">
@@ -3001,7 +3001,7 @@
         </is>
       </c>
       <c r="D147">
-        <v>23.90728367643491</v>
+        <v>24.16893739387245</v>
       </c>
     </row>
     <row r="148">
@@ -3019,7 +3019,7 @@
         </is>
       </c>
       <c r="D148">
-        <v>40.07822564720479</v>
+        <v>40.42331576276999</v>
       </c>
     </row>
     <row r="149">
@@ -3037,7 +3037,7 @@
         </is>
       </c>
       <c r="D149">
-        <v>50.98088761277739</v>
+        <v>51.40057383551586</v>
       </c>
     </row>
     <row r="150">
@@ -3055,7 +3055,7 @@
         </is>
       </c>
       <c r="D150">
-        <v>26.43269578972392</v>
+        <v>26.87525132577819</v>
       </c>
     </row>
     <row r="151">
@@ -3073,7 +3073,7 @@
         </is>
       </c>
       <c r="D151">
-        <v>40.195411101496</v>
+        <v>40.44744386907346</v>
       </c>
     </row>
     <row r="152">
@@ -3091,7 +3091,7 @@
         </is>
       </c>
       <c r="D152">
-        <v>44.4607497176964</v>
+        <v>44.81493990966285</v>
       </c>
     </row>
     <row r="153">
@@ -3109,7 +3109,7 @@
         </is>
       </c>
       <c r="D153">
-        <v>22.68134079209447</v>
+        <v>23.03913415628512</v>
       </c>
     </row>
     <row r="154">
@@ -3127,7 +3127,7 @@
         </is>
       </c>
       <c r="D154">
-        <v>35.40056423464949</v>
+        <v>35.80999827275107</v>
       </c>
     </row>
     <row r="155">
@@ -3145,7 +3145,7 @@
         </is>
       </c>
       <c r="D155">
-        <v>48.5813273640311</v>
+        <v>48.83835566942336</v>
       </c>
     </row>
     <row r="156">
@@ -3163,7 +3163,7 @@
         </is>
       </c>
       <c r="D156">
-        <v>24.07522580750063</v>
+        <v>24.17522336853573</v>
       </c>
     </row>
     <row r="157">
@@ -3181,7 +3181,7 @@
         </is>
       </c>
       <c r="D157">
-        <v>44.73660976961507</v>
+        <v>44.99395372707301</v>
       </c>
     </row>
     <row r="158">
@@ -3199,7 +3199,7 @@
         </is>
       </c>
       <c r="D158">
-        <v>50.72383921977751</v>
+        <v>50.95978819853207</v>
       </c>
     </row>
     <row r="159">
@@ -3217,7 +3217,7 @@
         </is>
       </c>
       <c r="D159">
-        <v>21.94518999858737</v>
+        <v>22.1911323126184</v>
       </c>
     </row>
     <row r="160">
@@ -3235,7 +3235,7 @@
         </is>
       </c>
       <c r="D160">
-        <v>42.65161935946987</v>
+        <v>42.90227029753969</v>
       </c>
     </row>
     <row r="161">
@@ -3253,7 +3253,7 @@
         </is>
       </c>
       <c r="D161">
-        <v>50.76793872329834</v>
+        <v>51.03322878869805</v>
       </c>
     </row>
     <row r="162">
@@ -3271,7 +3271,7 @@
         </is>
       </c>
       <c r="D162">
-        <v>24.09216602099994</v>
+        <v>24.28769183273082</v>
       </c>
     </row>
     <row r="163">
@@ -3289,7 +3289,7 @@
         </is>
       </c>
       <c r="D163">
-        <v>46.52641829877478</v>
+        <v>46.71273821640918</v>
       </c>
     </row>
     <row r="164">
@@ -3307,7 +3307,7 @@
         </is>
       </c>
       <c r="D164">
-        <v>51.90348025333653</v>
+        <v>52.2164730780087</v>
       </c>
     </row>
     <row r="165">
@@ -3325,7 +3325,7 @@
         </is>
       </c>
       <c r="D165">
-        <v>21.53385041102777</v>
+        <v>21.56473873800947</v>
       </c>
     </row>
     <row r="166">
@@ -3343,7 +3343,7 @@
         </is>
       </c>
       <c r="D166">
-        <v>46.62340314913844</v>
+        <v>46.95304035161302</v>
       </c>
     </row>
     <row r="167">
@@ -3361,7 +3361,7 @@
         </is>
       </c>
       <c r="D167">
-        <v>53.00737647680943</v>
+        <v>53.46671297696234</v>
       </c>
     </row>
     <row r="168">
@@ -3379,7 +3379,7 @@
         </is>
       </c>
       <c r="D168">
-        <v>22.06196376589551</v>
+        <v>22.08326949593994</v>
       </c>
     </row>
     <row r="169">
@@ -3397,7 +3397,7 @@
         </is>
       </c>
       <c r="D169">
-        <v>48.03920065184477</v>
+        <v>48.30224904845591</v>
       </c>
     </row>
     <row r="170">
@@ -3415,7 +3415,7 @@
         </is>
       </c>
       <c r="D170">
-        <v>50.98702502029055</v>
+        <v>51.30939582707289</v>
       </c>
     </row>
     <row r="171">
@@ -3433,7 +3433,7 @@
         </is>
       </c>
       <c r="D171">
-        <v>19.18539691371597</v>
+        <v>19.3904611477315</v>
       </c>
     </row>
     <row r="172">
@@ -3451,7 +3451,7 @@
         </is>
       </c>
       <c r="D172">
-        <v>43.65254440560215</v>
+        <v>44.04619589038061</v>
       </c>
     </row>
     <row r="173">
@@ -3469,7 +3469,7 @@
         </is>
       </c>
       <c r="D173">
-        <v>45.44769582155597</v>
+        <v>45.9729926228875</v>
       </c>
     </row>
     <row r="174">
@@ -3487,7 +3487,7 @@
         </is>
       </c>
       <c r="D174">
-        <v>16.11358900266058</v>
+        <v>16.26471652852506</v>
       </c>
     </row>
     <row r="175">
@@ -3505,7 +3505,7 @@
         </is>
       </c>
       <c r="D175">
-        <v>38.53350729735391</v>
+        <v>38.87786747669433</v>
       </c>
     </row>
     <row r="176">
@@ -3523,7 +3523,7 @@
         </is>
       </c>
       <c r="D176">
-        <v>47.29183402437114</v>
+        <v>47.61653690898133</v>
       </c>
     </row>
     <row r="177">
@@ -3541,7 +3541,7 @@
         </is>
       </c>
       <c r="D177">
-        <v>17.57331816596642</v>
+        <v>17.67378813291927</v>
       </c>
     </row>
     <row r="178">
@@ -3559,7 +3559,7 @@
         </is>
       </c>
       <c r="D178">
-        <v>38.25345287396197</v>
+        <v>38.85937714562419</v>
       </c>
     </row>
     <row r="179">
@@ -3577,7 +3577,7 @@
         </is>
       </c>
       <c r="D179">
-        <v>45.32445552365912</v>
+        <v>45.68699964722047</v>
       </c>
     </row>
     <row r="180">
@@ -3595,7 +3595,7 @@
         </is>
       </c>
       <c r="D180">
-        <v>18.13967226169456</v>
+        <v>18.33108683661714</v>
       </c>
     </row>
     <row r="181">
@@ -3613,7 +3613,7 @@
         </is>
       </c>
       <c r="D181">
-        <v>37.34529162595338</v>
+        <v>37.67264428543278</v>
       </c>
     </row>
     <row r="182">
@@ -3631,7 +3631,7 @@
         </is>
       </c>
       <c r="D182">
-        <v>44.30508051288648</v>
+        <v>44.64365618917876</v>
       </c>
     </row>
     <row r="183">
@@ -3649,7 +3649,7 @@
         </is>
       </c>
       <c r="D183">
-        <v>17.279721737399</v>
+        <v>17.56501557138101</v>
       </c>
     </row>
     <row r="184">
@@ -3667,7 +3667,7 @@
         </is>
       </c>
       <c r="D184">
-        <v>33.56102093160164</v>
+        <v>33.74984092562148</v>
       </c>
     </row>
     <row r="185">
@@ -3685,7 +3685,7 @@
         </is>
       </c>
       <c r="D185">
-        <v>35.94484139226011</v>
+        <v>36.30042301127871</v>
       </c>
     </row>
     <row r="186">
@@ -3703,7 +3703,7 @@
         </is>
       </c>
       <c r="D186">
-        <v>11.09580127837103</v>
+        <v>11.29432987031573</v>
       </c>
     </row>
     <row r="187">
@@ -3721,7 +3721,7 @@
         </is>
       </c>
       <c r="D187">
-        <v>25.662423500612</v>
+        <v>25.78002447980416</v>
       </c>
     </row>
     <row r="188">
@@ -3739,7 +3739,7 @@
         </is>
       </c>
       <c r="D188">
-        <v>38.74579717682061</v>
+        <v>39.16672821159747</v>
       </c>
     </row>
     <row r="189">
@@ -3757,7 +3757,7 @@
         </is>
       </c>
       <c r="D189">
-        <v>14.96752585485076</v>
+        <v>15.10864048260233</v>
       </c>
     </row>
     <row r="190">
@@ -3775,7 +3775,7 @@
         </is>
       </c>
       <c r="D190">
-        <v>29.68777685934803</v>
+        <v>29.89788640233279</v>
       </c>
     </row>
     <row r="191">
@@ -3793,7 +3793,7 @@
         </is>
       </c>
       <c r="D191">
-        <v>40.49692263948572</v>
+        <v>40.73357512115312</v>
       </c>
     </row>
     <row r="192">
@@ -3811,7 +3811,7 @@
         </is>
       </c>
       <c r="D192">
-        <v>17.91118825216415</v>
+        <v>18.20544404318655</v>
       </c>
     </row>
     <row r="193">
@@ -3829,7 +3829,7 @@
         </is>
       </c>
       <c r="D193">
-        <v>33.25348582061913</v>
+        <v>33.27569803763798</v>
       </c>
     </row>
     <row r="194">
@@ -3847,7 +3847,7 @@
         </is>
       </c>
       <c r="D194">
-        <v>42.05390129063226</v>
+        <v>42.24108701475445</v>
       </c>
     </row>
     <row r="195">
@@ -3865,7 +3865,7 @@
         </is>
       </c>
       <c r="D195">
-        <v>14.01284570398962</v>
+        <v>14.00057471710715</v>
       </c>
     </row>
     <row r="196">
@@ -3883,7 +3883,7 @@
         </is>
       </c>
       <c r="D196">
-        <v>29.86111559317002</v>
+        <v>30.05663068623446</v>
       </c>
     </row>
     <row r="197">
@@ -3901,7 +3901,7 @@
         </is>
       </c>
       <c r="D197">
-        <v>37.56926876987923</v>
+        <v>37.79433915523112</v>
       </c>
     </row>
     <row r="198">
@@ -3919,7 +3919,7 @@
         </is>
       </c>
       <c r="D198">
-        <v>15.29902916445127</v>
+        <v>15.29635662382162</v>
       </c>
     </row>
     <row r="199">
@@ -3937,7 +3937,7 @@
         </is>
       </c>
       <c r="D199">
-        <v>29.92474520986942</v>
+        <v>29.97265365193637</v>
       </c>
     </row>
   </sheetData>

</xml_diff>